<commit_message>
add Neil to names list
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Result" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$C$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$C$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,6 +521,23 @@
         </is>
       </c>
     </row>
+    <row r="6" hidden="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Neil</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KL</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
       <c r="I9" t="inlineStr">
         <is>
@@ -536,7 +553,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C5">
+  <autoFilter ref="A1:C6">
     <filterColumn colId="1" hiddenButton="0" showButton="1">
       <filters blank="0">
         <filter val="G"/>

</xml_diff>

<commit_message>
clear filter, show full names list
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -10,9 +10,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Result" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$C$6</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -453,7 +451,7 @@
         </is>
       </c>
     </row>
-    <row r="2" hidden="1">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>Ajay</t>
@@ -470,7 +468,7 @@
         </is>
       </c>
     </row>
-    <row r="3" hidden="1">
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>Bobby</t>
@@ -487,7 +485,7 @@
         </is>
       </c>
     </row>
-    <row r="4" hidden="1">
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>Heyna</t>
@@ -521,7 +519,7 @@
         </is>
       </c>
     </row>
-    <row r="6" hidden="1">
+    <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>Neil</t>
@@ -553,18 +551,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C6">
-    <filterColumn colId="1" hiddenButton="0" showButton="1">
-      <filters blank="0">
-        <filter val="G"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="2" hiddenButton="0" showButton="1">
-      <filters blank="0">
-        <filter val="TN"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>